<commit_message>
Daily NSE scan: 2026-10-11
</commit_message>
<xml_diff>
--- a/output/2026-10-11/enriched_analysis.xlsx
+++ b/output/2026-10-11/enriched_analysis.xlsx
@@ -2981,7 +2981,7 @@
         <v>4.5</v>
       </c>
       <c r="L11" t="n">
-        <v>62.09</v>
+        <v>61.84</v>
       </c>
       <c r="M11" t="n">
         <v>3.06</v>
@@ -4429,7 +4429,7 @@
         <v>7.91</v>
       </c>
       <c r="AD17" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AE17" t="b">
         <v>0</v>
@@ -12122,7 +12122,7 @@
         <v>4.5</v>
       </c>
       <c r="F11" t="n">
-        <v>62.09</v>
+        <v>61.84</v>
       </c>
       <c r="G11" t="n">
         <v>3.06</v>

</xml_diff>